<commit_message>
Update soccer trades 2026-08-08 21:02:18 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Primera Nacional/trades.xlsx
+++ b/data/sxbet/ligas/Primera Nacional/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V24"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x0a5de930b5a6b8aca1699b666034af3891a3aa920021791d6d13e0297fb7903f</t>
+          <t>0x86f4b24298f4c19f9f856cb19af2a260f24dc2d391f252248469436057ea1d1a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>49.99999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Almirante Brown -1</t>
+          <t>Deportivo Moron -1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Deportivo Moron vs Acassuso</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Deportivo Moron</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Acassuso</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
+          <t>0xb61b063252c01d0525ae633a0276dc1830eabd418482fddec925fcbd602a2a75</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683452</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786218515</t>
+          <t>1786220171</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786298400</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>80.971644</t>
+          <t>1.900238</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,23 +643,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x17d5a08f8fa305f31f27442393c64f497dd3893417da6e76c321c4c2a187320d</t>
+          <t>0x0a5de930b5a6b8aca1699b666034af3891a3aa920021791d6d13e0297fb7903f</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>49.18897</t>
+          <t>49.99999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4737</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -667,7 +671,11 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Almirante Brown -1</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -720,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786218084</t>
+          <t>1786218515</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>103.82896</t>
+          <t>80.971644</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,28 +755,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x56975f372357be259365cb7d2929c88d4fae157eea7a71d53d57cb234834f2ca</t>
+          <t>0x17d5a08f8fa305f31f27442393c64f497dd3893417da6e76c321c4c2a187320d</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>49.18897</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4812</t>
+          <t>1.4737</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -779,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Club Atletico Mitre de Santiago del Estero vs Defensores de Belgrano Buenos Aires</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Club Atletico Mitre de Santiago del Estero</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Defensores de Belgrano Buenos Aires</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xa8ade64a3adb0ea38de67a61105ef31beb490d5a7287715b76ae124536d359cc</t>
+          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19683493</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786215674</t>
+          <t>1786218084</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2.077922</t>
+          <t>103.82896</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,7 +859,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xff53df1f3446908699196d44fcdb8b39c1bd15c7ed519f0d730e55a51a6eb38f</t>
+          <t>0x56975f372357be259365cb7d2929c88d4fae157eea7a71d53d57cb234834f2ca</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -859,11 +867,7 @@
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>1</t>
@@ -871,19 +875,15 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.3713</t>
+          <t>1.4812</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Almirante Brown</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -891,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Club Atletico Mitre de Santiago del Estero vs Defensores de Belgrano Buenos Aires</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Club Atletico Mitre de Santiago del Estero</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Defensores de Belgrano Buenos Aires</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x63a8bf73c1084ef223fdd1096dccd16232e7a455fad77f7f0891be1588ebeb88</t>
+          <t>0xa8ade64a3adb0ea38de67a61105ef31beb490d5a7287715b76ae124536d359cc</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683493</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -936,17 +936,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786215673</t>
+          <t>1786215674</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2.693603</t>
+          <t>2.077922</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,12 +963,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x249d52552e7acb9f472d2a4c48ab754622ba572903281739a3e10b4d509dccb0</t>
+          <t>0xff53df1f3446908699196d44fcdb8b39c1bd15c7ed519f0d730e55a51a6eb38f</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -978,22 +978,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.2288</t>
+          <t>1.3713</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Almirante Brown -1</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
+          <t>0x63a8bf73c1084ef223fdd1096dccd16232e7a455fad77f7f0891be1588ebeb88</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786214209</t>
+          <t>1786215673</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>6.295082</t>
+          <t>2.693603</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,12 +1075,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xf65c55196eeb0d21e7e3866ad26f8c3f2fee2aef273ddde5423e31fb40a51469</t>
+          <t>0x249d52552e7acb9f472d2a4c48ab754622ba572903281739a3e10b4d509dccb0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1090,39 +1090,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>121.81</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4363</t>
+          <t>1.2288</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>Almirante Brown -1</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>Almirante Brown</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Almirante Brown</t>
-        </is>
-      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>Ciudad Bolivar</t>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x63a8bf73c1084ef223fdd1096dccd16232e7a455fad77f7f0891be1588ebeb88</t>
+          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786213844</t>
+          <t>1786214209</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>279.22063</t>
+          <t>6.295082</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x1bb20a2bf22e4fe06b44c06b9c2caa21f3f2a7c9d0cce1a2346f79e76022cd1f</t>
+          <t>0xf65c55196eeb0d21e7e3866ad26f8c3f2fee2aef273ddde5423e31fb40a51469</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>21.05</t>
+          <t>121.81</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Almirante Brown -0.5</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xfa00d2f0c7b5053ee336b303a0e7ad9cec0b8d539367773b7efee5c86cb2b59d</t>
+          <t>0x63a8bf73c1084ef223fdd1096dccd16232e7a455fad77f7f0891be1588ebeb88</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786213843</t>
+          <t>1786213844</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>48.252149</t>
+          <t>279.22063</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,7 +1299,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xc51052f8e449b4d56cc87b697bfc8eb0d3a88ae218dee1da3d725fa94163bc75</t>
+          <t>0x1bb20a2bf22e4fe06b44c06b9c2caa21f3f2a7c9d0cce1a2346f79e76022cd1f</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1307,28 +1307,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>77.29513</t>
+          <t>21.05</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.2588</t>
+          <t>1.4363</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Almirante Brown -0.5</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>Almirante Brown vs Ciudad Bolivar</t>
@@ -1346,7 +1354,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xaa5316c6f6544d74142ad6db34a3745918f237ffb1a657e000693947e81b65d6</t>
+          <t>0xfa00d2f0c7b5053ee336b303a0e7ad9cec0b8d539367773b7efee5c86cb2b59d</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1376,7 +1384,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786212849</t>
+          <t>1786213843</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1386,7 +1394,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>298.72514</t>
+          <t>48.252149</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,7 +1411,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x0aeb4fe40f7d734cf244c144e6c064568b40b222193c9f93c641d1b31af3752e</t>
+          <t>0xc51052f8e449b4d56cc87b697bfc8eb0d3a88ae218dee1da3d725fa94163bc75</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1414,7 +1422,7 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16.89162</t>
+          <t>77.29513</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1480,7 +1488,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786212805</t>
+          <t>1786212849</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1490,7 +1498,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>65.281623</t>
+          <t>298.72514</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,7 +1515,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x383b895a5fe529a887369a0f113c516fdc7f6125d54381acf9695997ef22d039</t>
+          <t>0x0aeb4fe40f7d734cf244c144e6c064568b40b222193c9f93c641d1b31af3752e</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1515,19 +1523,15 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.26905</t>
+          <t>16.89162</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.2588</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1535,26 +1539,22 @@
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>Almirante Brown</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Almirante Brown</t>
-        </is>
-      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>Ciudad Bolivar</t>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786211779</t>
+          <t>1786212805</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>15.126242</t>
+          <t>65.281623</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,12 +1619,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xcfb6add6f8610a64ffc187beb9e16bf2bacb27b54a0f0aaefa6bfb437239b893</t>
+          <t>0x383b895a5fe529a887369a0f113c516fdc7f6125d54381acf9695997ef22d039</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>24.89998</t>
+          <t>11.26905</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786211777</t>
+          <t>1786211779</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>33.422792</t>
+          <t>15.126242</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,12 +1731,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xd41652604437a4e92e0d78b653d4d49d8dedd2e153d1340dad89b9b93e182a48</t>
+          <t>0xcfb6add6f8610a64ffc187beb9e16bf2bacb27b54a0f0aaefa6bfb437239b893</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1746,22 +1746,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>24.89998</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.4163</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Primera Nacional</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Atl. Rafaela</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1771,27 +1771,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Atl. Rafaela vs Chacarita Juniors</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Atl. Rafaela</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Chacarita Juniors</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xe738e9ba05492fab73eaaf6da211b84caadc72b08b26f1cd30fa8737e283bb44</t>
+          <t>0xaa5316c6f6544d74142ad6db34a3745918f237ffb1a657e000693947e81b65d6</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19683450</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1816,17 +1816,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786211028</t>
+          <t>1786211777</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786215600</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2.402402</t>
+          <t>33.422792</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1843,31 +1843,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x562fd7c6419c807ed04d3cacac95f861805f96704bd535e265399fb9d2c2b609</t>
+          <t>0xd41652604437a4e92e0d78b653d4d49d8dedd2e153d1340dad89b9b93e182a48</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>5.32</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.405</t>
+          <t>1.4163</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Atl. Rafaela</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -1875,27 +1883,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
+          <t>Atl. Rafaela vs Chacarita Juniors</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros</t>
+          <t>Atl. Rafaela</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Chacarita Juniors</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
+          <t>0xe738e9ba05492fab73eaaf6da211b84caadc72b08b26f1cd30fa8737e283bb44</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19683453</t>
+          <t>L19683450</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1920,17 +1928,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786210845</t>
+          <t>1786211028</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786215600</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>13.135802</t>
+          <t>2.402402</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,39 +1955,31 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x0bb7a6822220bf40d7b279f99a54f46025f393ba95bb38b6d6dc98192886b3ed</t>
+          <t>0x562fd7c6419c807ed04d3cacac95f861805f96704bd535e265399fb9d2c2b609</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.99999</t>
+          <t>5.32</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.405</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Agropecuario</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -1987,27 +1987,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Agropecuario vs Atletico Guemes</t>
+          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Agropecuario</t>
+          <t>Estudiantes de Caseros</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Atletico Guemes</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xae66c7fab3c9c76fbc29d9e9778ef4845d8a6b8d092cff34320f100020113c49</t>
+          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19683451</t>
+          <t>L19683453</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786205982</t>
+          <t>1786210845</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1.814041</t>
+          <t>13.135802</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2059,7 +2059,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xe17b2546f4b90c8647ba975c279e39dec1fda5a003adfb8a2b39bb12a3519b10</t>
+          <t>0x0bb7a6822220bf40d7b279f99a54f46025f393ba95bb38b6d6dc98192886b3ed</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2074,12 +2074,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.99999</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.3613</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Agropecuario</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2099,27 +2099,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Agropecuario vs Atletico Guemes</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Agropecuario</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Atletico Guemes</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xd5906ce08d61f7c5ee45fcebd2c8baeed5558387398ea332817a4b632f439b6d</t>
+          <t>0xae66c7fab3c9c76fbc29d9e9778ef4845d8a6b8d092cff34320f100020113c49</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683451</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786205963</t>
+          <t>1786205982</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2.768166</t>
+          <t>1.814041</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2171,7 +2171,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xcfe218822e89cbef5841f3045f551cc65acf353d8e240f943e2b61c54ea79a68</t>
+          <t>0xe17b2546f4b90c8647ba975c279e39dec1fda5a003adfb8a2b39bb12a3519b10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.3337</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2211,27 +2211,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xf238b96ec9e2421db79973de945f1fc0c3f8bb99c31cda32d011ebaabfd2db86</t>
+          <t>0xd5906ce08d61f7c5ee45fcebd2c8baeed5558387398ea332817a4b632f439b6d</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19683453</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786205938</t>
+          <t>1786205963</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2.996255</t>
+          <t>2.768166</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2283,31 +2283,39 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x1b9fcb29010a212f74af57040114154e78748f06a4d826be4397ddadb45ac31b</t>
+          <t>0xcfe218822e89cbef5841f3045f551cc65acf353d8e240f943e2b61c54ea79a68</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>21.69</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.3337</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2315,27 +2323,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Estudiantes de Caseros</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
+          <t>0xf238b96ec9e2421db79973de945f1fc0c3f8bb99c31cda32d011ebaabfd2db86</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683453</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2360,7 +2368,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786190525</t>
+          <t>1786205938</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2370,7 +2378,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>48.066482</t>
+          <t>2.996255</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2387,23 +2395,23 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x3177792dd6a7185e37ae06612104cf5a35d137d7f535a889a83a7e9b7c174506</t>
+          <t>0x1b9fcb29010a212f74af57040114154e78748f06a4d826be4397ddadb45ac31b</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>18.35495</t>
+          <t>21.69</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.4963</t>
+          <t>1.4512</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2464,7 +2472,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786190491</t>
+          <t>1786190525</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2474,7 +2482,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>36.987305</t>
+          <t>48.066482</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,7 +2499,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x54ed4ee2a6ebdab49498137f1accea542ead806f21430a0a771cc4872a044e43</t>
+          <t>0x3177792dd6a7185e37ae06612104cf5a35d137d7f535a889a83a7e9b7c174506</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2499,19 +2507,15 @@
           <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>20.10741</t>
+          <t>18.35495</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.4963</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2519,11 +2523,7 @@
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786190485</t>
+          <t>1786190491</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>36.979145</t>
+          <t>36.987305</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,23 +2603,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x544fe5c906328d009917b591611ff3438cef85f8b42d9f67732cbbd5eabbb8dd</t>
+          <t>0x54ed4ee2a6ebdab49498137f1accea542ead806f21430a0a771cc4872a044e43</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>21.69</t>
+          <t>20.10741</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2627,7 +2631,11 @@
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2690,7 +2698,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>48.066482</t>
+          <t>36.979145</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2707,7 +2715,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xb2f3ea804e1760a01d3a93678f0e2119f1ea2a9db0dc4711a06cc7bcba42b0c2</t>
+          <t>0x544fe5c906328d009917b591611ff3438cef85f8b42d9f67732cbbd5eabbb8dd</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2718,12 +2726,12 @@
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>17.47</t>
+          <t>21.69</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.405</t>
+          <t>1.4512</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2739,27 +2747,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
+          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19683453</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2784,7 +2792,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786190461</t>
+          <t>1786190485</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2794,7 +2802,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>43.135802</t>
+          <t>48.066482</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2811,7 +2819,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xa7eafbb77d425fc2347b4ee3e4f4e1b85f6d0f81420605db76ebfeeaa793a428</t>
+          <t>0xb2f3ea804e1760a01d3a93678f0e2119f1ea2a9db0dc4711a06cc7bcba42b0c2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2822,12 +2830,12 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>21.69</t>
+          <t>17.47</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.405</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2843,27 +2851,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Estudiantes de Caseros</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
+          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683453</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2888,7 +2896,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786190458</t>
+          <t>1786190461</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2898,7 +2906,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>48.066482</t>
+          <t>43.135802</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2915,110 +2923,214 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>0xa7eafbb77d425fc2347b4ee3e4f4e1b85f6d0f81420605db76ebfeeaa793a428</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>21.69</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Almirante Brown</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>L19683447</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1786190458</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>48.066482</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>0x5c5b512ea725fac30531bf5fe91f34f3ccc0eeff23890c18f25c3f329007c589</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>1.3638</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>Almirante Brown</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>Ciudad Bolivar</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>0xd5906ce08d61f7c5ee45fcebd2c8baeed5558387398ea332817a4b632f439b6d</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>L19683447</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
         <is>
           <t>1786125660</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="S25" t="inlineStr">
         <is>
           <t>1786212000</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
+      <c r="T25" t="inlineStr">
         <is>
           <t>2.749141</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="U25" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr">
+      <c r="V25" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-09 03:02:13 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Primera Nacional/trades.xlsx
+++ b/data/sxbet/ligas/Primera Nacional/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V26"/>
+  <dimension ref="A1:V28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,15 +531,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xd3b94d194e43cc84f0a1b82723594ea6689a6aa2a4a7dccbc8a3d19fc321e49b</t>
+          <t>0x4e811c319e5e3a1fc1968ce0f31b4c15eb7222daa616252d99f9abc611408746</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>1</t>
@@ -547,15 +551,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5238</t>
+          <t>1.2925</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Deportivo Moron vs Acassuso</t>
+          <t>Colon de Santa Fe vs San Telmo</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Deportivo Moron</t>
+          <t>Colon de Santa Fe</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Acassuso</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x108eaba0441fb45ec8e0073e945ae0ac1e138c933e4f2839816cd3198d7dd4d2</t>
+          <t>0x2e49527408facf21253a0a1eafe51280b82e4c31919e91a396332f19ec366401</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19683452</t>
+          <t>L19683494</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786225000</t>
+          <t>1786243741</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786298400</t>
+          <t>1786300200</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.909308</t>
+          <t>3.418803</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x86f4b24298f4c19f9f856cb19af2a260f24dc2d391f252248469436057ea1d1a</t>
+          <t>0xb8631aeb398192a03386505542f05fa15e34db501204baa8745a4d4b5c1651b7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -650,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.99999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.6538</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Deportivo Moron -1</t>
+          <t>Deportivo Moron</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -690,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xb61b063252c01d0525ae633a0276dc1830eabd418482fddec925fcbd602a2a75</t>
+          <t>0x7514a255ce41be3c5db9f8849ba04e78dab80f02d1fe78c2aae82bbc843a9745</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786220171</t>
+          <t>1786243225</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.900238</t>
+          <t>1.529621</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,39 +755,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x0a5de930b5a6b8aca1699b666034af3891a3aa920021791d6d13e0297fb7903f</t>
+          <t>0xd3b94d194e43cc84f0a1b82723594ea6689a6aa2a4a7dccbc8a3d19fc321e49b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>49.99999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.5238</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Almirante Brown -1</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -787,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Deportivo Moron vs Acassuso</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Deportivo Moron</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Acassuso</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
+          <t>0x108eaba0441fb45ec8e0073e945ae0ac1e138c933e4f2839816cd3198d7dd4d2</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683452</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786218515</t>
+          <t>1786225000</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786298400</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>80.971644</t>
+          <t>1.909308</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,23 +859,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x17d5a08f8fa305f31f27442393c64f497dd3893417da6e76c321c4c2a187320d</t>
+          <t>0x86f4b24298f4c19f9f856cb19af2a260f24dc2d391f252248469436057ea1d1a</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>49.18897</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.4737</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -883,7 +887,11 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Deportivo Moron -1</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -891,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Deportivo Moron vs Acassuso</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Deportivo Moron</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Acassuso</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
+          <t>0xb61b063252c01d0525ae633a0276dc1830eabd418482fddec925fcbd602a2a75</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683452</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -936,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786218084</t>
+          <t>1786220171</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786298400</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>103.82896</t>
+          <t>1.900238</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,31 +971,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x56975f372357be259365cb7d2929c88d4fae157eea7a71d53d57cb234834f2ca</t>
+          <t>0x0a5de930b5a6b8aca1699b666034af3891a3aa920021791d6d13e0297fb7903f</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>49.99999</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.4812</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Almirante Brown -1</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -995,27 +1011,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Club Atletico Mitre de Santiago del Estero vs Defensores de Belgrano Buenos Aires</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Club Atletico Mitre de Santiago del Estero</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Defensores de Belgrano Buenos Aires</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xa8ade64a3adb0ea38de67a61105ef31beb490d5a7287715b76ae124536d359cc</t>
+          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19683493</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1040,17 +1056,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786215674</t>
+          <t>1786218515</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2.077922</t>
+          <t>80.971644</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,54 +1083,46 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xff53df1f3446908699196d44fcdb8b39c1bd15c7ed519f0d730e55a51a6eb38f</t>
+          <t>0x17d5a08f8fa305f31f27442393c64f497dd3893417da6e76c321c4c2a187320d</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>49.18897</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.3713</t>
+          <t>1.4737</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Almirante Brown</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Almirante Brown</t>
-        </is>
-      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>Ciudad Bolivar</t>
@@ -1122,7 +1130,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x63a8bf73c1084ef223fdd1096dccd16232e7a455fad77f7f0891be1588ebeb88</t>
+          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786215673</t>
+          <t>1786218084</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2.693603</t>
+          <t>103.82896</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,39 +1187,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x249d52552e7acb9f472d2a4c48ab754622ba572903281739a3e10b4d509dccb0</t>
+          <t>0x56975f372357be259365cb7d2929c88d4fae157eea7a71d53d57cb234834f2ca</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2288</t>
+          <t>1.4812</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Almirante Brown -1</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -1219,27 +1219,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Club Atletico Mitre de Santiago del Estero vs Defensores de Belgrano Buenos Aires</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Club Atletico Mitre de Santiago del Estero</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Defensores de Belgrano Buenos Aires</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
+          <t>0xa8ade64a3adb0ea38de67a61105ef31beb490d5a7287715b76ae124536d359cc</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683493</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1264,17 +1264,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786214209</t>
+          <t>1786215674</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>6.295082</t>
+          <t>2.077922</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,12 +1291,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xf65c55196eeb0d21e7e3866ad26f8c3f2fee2aef273ddde5423e31fb40a51469</t>
+          <t>0xff53df1f3446908699196d44fcdb8b39c1bd15c7ed519f0d730e55a51a6eb38f</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1306,12 +1306,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>121.81</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.4363</t>
+          <t>1.3713</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786213844</t>
+          <t>1786215673</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>279.22063</t>
+          <t>2.693603</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,12 +1403,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x1bb20a2bf22e4fe06b44c06b9c2caa21f3f2a7c9d0cce1a2346f79e76022cd1f</t>
+          <t>0x249d52552e7acb9f472d2a4c48ab754622ba572903281739a3e10b4d509dccb0</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1418,22 +1418,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>21.05</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.4363</t>
+          <t>1.2288</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Almirante Brown -0.5</t>
+          <t>Almirante Brown -1</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xfa00d2f0c7b5053ee336b303a0e7ad9cec0b8d539367773b7efee5c86cb2b59d</t>
+          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786213843</t>
+          <t>1786214209</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>48.252149</t>
+          <t>6.295082</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1515,7 +1515,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xc51052f8e449b4d56cc87b697bfc8eb0d3a88ae218dee1da3d725fa94163bc75</t>
+          <t>0xf65c55196eeb0d21e7e3866ad26f8c3f2fee2aef273ddde5423e31fb40a51469</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1523,28 +1523,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>77.29513</t>
+          <t>121.81</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.2588</t>
+          <t>1.4363</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Almirante Brown</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>Almirante Brown vs Ciudad Bolivar</t>
@@ -1562,7 +1570,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xaa5316c6f6544d74142ad6db34a3745918f237ffb1a657e000693947e81b65d6</t>
+          <t>0x63a8bf73c1084ef223fdd1096dccd16232e7a455fad77f7f0891be1588ebeb88</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1592,7 +1600,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786212849</t>
+          <t>1786213844</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1602,7 +1610,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>298.72514</t>
+          <t>279.22063</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,7 +1627,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x0aeb4fe40f7d734cf244c144e6c064568b40b222193c9f93c641d1b31af3752e</t>
+          <t>0x1bb20a2bf22e4fe06b44c06b9c2caa21f3f2a7c9d0cce1a2346f79e76022cd1f</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1627,28 +1635,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>16.89162</t>
+          <t>21.05</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.2588</t>
+          <t>1.4363</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Almirante Brown -0.5</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>Almirante Brown vs Ciudad Bolivar</t>
@@ -1666,7 +1682,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xaa5316c6f6544d74142ad6db34a3745918f237ffb1a657e000693947e81b65d6</t>
+          <t>0xfa00d2f0c7b5053ee336b303a0e7ad9cec0b8d539367773b7efee5c86cb2b59d</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1696,7 +1712,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786212805</t>
+          <t>1786213843</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1706,7 +1722,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>65.281623</t>
+          <t>48.252149</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1723,7 +1739,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x383b895a5fe529a887369a0f113c516fdc7f6125d54381acf9695997ef22d039</t>
+          <t>0xc51052f8e449b4d56cc87b697bfc8eb0d3a88ae218dee1da3d725fa94163bc75</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1731,19 +1747,15 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11.26905</t>
+          <t>77.29513</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.2588</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1751,26 +1763,22 @@
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>Almirante Brown</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Almirante Brown</t>
-        </is>
-      </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>Ciudad Bolivar</t>
@@ -1808,7 +1816,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786211779</t>
+          <t>1786212849</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1818,7 +1826,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>15.126242</t>
+          <t>298.72514</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1835,27 +1843,23 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xcfb6add6f8610a64ffc187beb9e16bf2bacb27b54a0f0aaefa6bfb437239b893</t>
+          <t>0x0aeb4fe40f7d734cf244c144e6c064568b40b222193c9f93c641d1b31af3752e</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>24.89998</t>
+          <t>16.89162</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.2588</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1863,26 +1867,22 @@
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>Almirante Brown</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Almirante Brown</t>
-        </is>
-      </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>Ciudad Bolivar</t>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786211777</t>
+          <t>1786212805</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>33.422792</t>
+          <t>65.281623</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,12 +1947,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xd41652604437a4e92e0d78b653d4d49d8dedd2e153d1340dad89b9b93e182a48</t>
+          <t>0x383b895a5fe529a887369a0f113c516fdc7f6125d54381acf9695997ef22d039</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1962,22 +1962,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>11.26905</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.4163</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Primera Nacional</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Atl. Rafaela</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1987,27 +1987,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Atl. Rafaela vs Chacarita Juniors</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Atl. Rafaela</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Chacarita Juniors</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xe738e9ba05492fab73eaaf6da211b84caadc72b08b26f1cd30fa8737e283bb44</t>
+          <t>0xaa5316c6f6544d74142ad6db34a3745918f237ffb1a657e000693947e81b65d6</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19683450</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2032,17 +2032,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786211028</t>
+          <t>1786211779</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786215600</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2.402402</t>
+          <t>15.126242</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2059,7 +2059,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x562fd7c6419c807ed04d3cacac95f861805f96704bd535e265399fb9d2c2b609</t>
+          <t>0xcfb6add6f8610a64ffc187beb9e16bf2bacb27b54a0f0aaefa6bfb437239b893</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2067,23 +2067,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5.32</t>
+          <t>24.89998</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.405</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Almirante Brown</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2091,27 +2099,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
+          <t>0xaa5316c6f6544d74142ad6db34a3745918f237ffb1a657e000693947e81b65d6</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19683453</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2136,7 +2144,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786210845</t>
+          <t>1786211777</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2146,7 +2154,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>13.135802</t>
+          <t>33.422792</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2163,7 +2171,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x0bb7a6822220bf40d7b279f99a54f46025f393ba95bb38b6d6dc98192886b3ed</t>
+          <t>0xd41652604437a4e92e0d78b653d4d49d8dedd2e153d1340dad89b9b93e182a48</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2178,12 +2186,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.99999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.4163</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2193,7 +2201,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Agropecuario</t>
+          <t>Atl. Rafaela</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2203,27 +2211,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Agropecuario vs Atletico Guemes</t>
+          <t>Atl. Rafaela vs Chacarita Juniors</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Agropecuario</t>
+          <t>Atl. Rafaela</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Atletico Guemes</t>
+          <t>Chacarita Juniors</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xae66c7fab3c9c76fbc29d9e9778ef4845d8a6b8d092cff34320f100020113c49</t>
+          <t>0xe738e9ba05492fab73eaaf6da211b84caadc72b08b26f1cd30fa8737e283bb44</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19683451</t>
+          <t>L19683450</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2248,17 +2256,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786205982</t>
+          <t>1786211028</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786215600</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1.814041</t>
+          <t>2.402402</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2275,39 +2283,31 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xe17b2546f4b90c8647ba975c279e39dec1fda5a003adfb8a2b39bb12a3519b10</t>
+          <t>0x562fd7c6419c807ed04d3cacac95f861805f96704bd535e265399fb9d2c2b609</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5.32</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.3613</t>
+          <t>1.405</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2315,27 +2315,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Estudiantes de Caseros</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xd5906ce08d61f7c5ee45fcebd2c8baeed5558387398ea332817a4b632f439b6d</t>
+          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683453</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786205963</t>
+          <t>1786210845</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2.768166</t>
+          <t>13.135802</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xcfe218822e89cbef5841f3045f551cc65acf353d8e240f943e2b61c54ea79a68</t>
+          <t>0x0bb7a6822220bf40d7b279f99a54f46025f393ba95bb38b6d6dc98192886b3ed</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2402,12 +2402,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.99999</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.3337</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Agropecuario</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2427,27 +2427,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
+          <t>Agropecuario vs Atletico Guemes</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros</t>
+          <t>Agropecuario</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Atletico Guemes</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xf238b96ec9e2421db79973de945f1fc0c3f8bb99c31cda32d011ebaabfd2db86</t>
+          <t>0xae66c7fab3c9c76fbc29d9e9778ef4845d8a6b8d092cff34320f100020113c49</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19683453</t>
+          <t>L19683451</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786205938</t>
+          <t>1786205982</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2.996255</t>
+          <t>1.814041</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2499,31 +2499,39 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x1b9fcb29010a212f74af57040114154e78748f06a4d826be4397ddadb45ac31b</t>
+          <t>0xe17b2546f4b90c8647ba975c279e39dec1fda5a003adfb8a2b39bb12a3519b10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>21.69</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2546,7 +2554,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
+          <t>0xd5906ce08d61f7c5ee45fcebd2c8baeed5558387398ea332817a4b632f439b6d</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2576,7 +2584,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786190525</t>
+          <t>1786205963</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2586,7 +2594,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>48.066482</t>
+          <t>2.768166</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,31 +2611,39 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x3177792dd6a7185e37ae06612104cf5a35d137d7f535a889a83a7e9b7c174506</t>
+          <t>0xcfe218822e89cbef5841f3045f551cc65acf353d8e240f943e2b61c54ea79a68</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>18.35495</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.4963</t>
+          <t>1.3337</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2635,27 +2651,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Estudiantes de Caseros</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
+          <t>0xf238b96ec9e2421db79973de945f1fc0c3f8bb99c31cda32d011ebaabfd2db86</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683453</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2680,7 +2696,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786190491</t>
+          <t>1786205938</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2690,7 +2706,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>36.987305</t>
+          <t>2.996255</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2707,27 +2723,23 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x54ed4ee2a6ebdab49498137f1accea542ead806f21430a0a771cc4872a044e43</t>
+          <t>0x1b9fcb29010a212f74af57040114154e78748f06a4d826be4397ddadb45ac31b</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>20.10741</t>
+          <t>21.69</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.4512</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2735,11 +2747,7 @@
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2792,7 +2800,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786190485</t>
+          <t>1786190525</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2802,7 +2810,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>36.979145</t>
+          <t>48.066482</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2819,23 +2827,23 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x544fe5c906328d009917b591611ff3438cef85f8b42d9f67732cbbd5eabbb8dd</t>
+          <t>0x3177792dd6a7185e37ae06612104cf5a35d137d7f535a889a83a7e9b7c174506</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>21.69</t>
+          <t>18.35495</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.4963</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2896,7 +2904,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786190485</t>
+          <t>1786190491</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2906,7 +2914,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>48.066482</t>
+          <t>36.987305</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2923,23 +2931,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xb2f3ea804e1760a01d3a93678f0e2119f1ea2a9db0dc4711a06cc7bcba42b0c2</t>
+          <t>0x54ed4ee2a6ebdab49498137f1accea542ead806f21430a0a771cc4872a044e43</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>17.47</t>
+          <t>20.10741</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.405</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2947,7 +2959,11 @@
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2955,27 +2971,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
+          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19683453</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3000,7 +3016,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786190461</t>
+          <t>1786190485</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3010,7 +3026,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>43.135802</t>
+          <t>36.979145</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3027,7 +3043,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xa7eafbb77d425fc2347b4ee3e4f4e1b85f6d0f81420605db76ebfeeaa793a428</t>
+          <t>0x544fe5c906328d009917b591611ff3438cef85f8b42d9f67732cbbd5eabbb8dd</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3104,7 +3120,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786190458</t>
+          <t>1786190485</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3131,110 +3147,318 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>0xb2f3ea804e1760a01d3a93678f0e2119f1ea2a9db0dc4711a06cc7bcba42b0c2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>17.47</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.405</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Estudiantes de Caseros</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Deportivo Madryn</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>L19683453</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1786190461</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>43.135802</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>0xa7eafbb77d425fc2347b4ee3e4f4e1b85f6d0f81420605db76ebfeeaa793a428</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>21.69</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Almirante Brown</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>L19683447</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1786190458</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>48.066482</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>0x5c5b512ea725fac30531bf5fe91f34f3ccc0eeff23890c18f25c3f329007c589</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>1.3638</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>Almirante Brown</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Ciudad Bolivar</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>0xd5906ce08d61f7c5ee45fcebd2c8baeed5558387398ea332817a4b632f439b6d</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>L19683447</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
         <is>
           <t>1786125660</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="S28" t="inlineStr">
         <is>
           <t>1786212000</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="T28" t="inlineStr">
         <is>
           <t>2.749141</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="U28" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr">
+      <c r="V28" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-09 11:02:44 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Primera Nacional/trades.xlsx
+++ b/data/sxbet/ligas/Primera Nacional/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V29"/>
+  <dimension ref="A1:V30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x2121e08c4ea1fe2d49a3bb388fba9e232ef9c06335c04e5eae0bf7766975512a</t>
+          <t>0x0847a2541998eecfe02d138796b14ef3d6719061787498f4888f6e14c0d196ff</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>30.06</t>
+          <t>38.54</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.6262</t>
+          <t>1.125</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Colon de Santa Fe</t>
+          <t>Club Almagro</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Colon de Santa Fe vs San Telmo</t>
+          <t>Quilmes vs Club Almagro</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Colon de Santa Fe</t>
+          <t>Quilmes</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Club Almagro</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x1a11ec80edeaae24566c4f4f891cc2afc56b377b24997a6e8ee533eeaaad5c92</t>
+          <t>0x03ed0858b563c1becf38b195ad94b1a84eb89c3ca8ca10b1a34220bff142f9b2</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19683494</t>
+          <t>L19683499</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786253941</t>
+          <t>1786270828</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786300200</t>
+          <t>1786305600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>308.32</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x4e811c319e5e3a1fc1968ce0f31b4c15eb7222daa616252d99f9abc611408746</t>
+          <t>0x2121e08c4ea1fe2d49a3bb388fba9e232ef9c06335c04e5eae0bf7766975512a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>30.06</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.2925</t>
+          <t>1.6262</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Colon de Santa Fe</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x2e49527408facf21253a0a1eafe51280b82e4c31919e91a396332f19ec366401</t>
+          <t>0x1a11ec80edeaae24566c4f4f891cc2afc56b377b24997a6e8ee533eeaaad5c92</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786243741</t>
+          <t>1786253941</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>3.418803</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xb8631aeb398192a03386505542f05fa15e34db501204baa8745a4d4b5c1651b7</t>
+          <t>0x4e811c319e5e3a1fc1968ce0f31b4c15eb7222daa616252d99f9abc611408746</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.99999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.6538</t>
+          <t>1.2925</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Deportivo Moron</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -795,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Deportivo Moron vs Acassuso</t>
+          <t>Colon de Santa Fe vs San Telmo</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Deportivo Moron</t>
+          <t>Colon de Santa Fe</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Acassuso</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x7514a255ce41be3c5db9f8849ba04e78dab80f02d1fe78c2aae82bbc843a9745</t>
+          <t>0x2e49527408facf21253a0a1eafe51280b82e4c31919e91a396332f19ec366401</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19683452</t>
+          <t>L19683494</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,17 +840,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786243225</t>
+          <t>1786243741</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786298400</t>
+          <t>1786300200</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1.529621</t>
+          <t>3.418803</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,31 +867,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xd3b94d194e43cc84f0a1b82723594ea6689a6aa2a4a7dccbc8a3d19fc321e49b</t>
+          <t>0xb8631aeb398192a03386505542f05fa15e34db501204baa8745a4d4b5c1651b7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.99999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.5238</t>
+          <t>1.6538</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Deportivo Moron</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -914,7 +922,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x108eaba0441fb45ec8e0073e945ae0ac1e138c933e4f2839816cd3198d7dd4d2</t>
+          <t>0x7514a255ce41be3c5db9f8849ba04e78dab80f02d1fe78c2aae82bbc843a9745</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786225000</t>
+          <t>1786243225</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1.909308</t>
+          <t>1.529621</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x86f4b24298f4c19f9f856cb19af2a260f24dc2d391f252248469436057ea1d1a</t>
+          <t>0xd3b94d194e43cc84f0a1b82723594ea6689a6aa2a4a7dccbc8a3d19fc321e49b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -979,11 +987,7 @@
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>1</t>
@@ -991,19 +995,15 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.5238</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Deportivo Moron -1</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xb61b063252c01d0525ae633a0276dc1830eabd418482fddec925fcbd602a2a75</t>
+          <t>0x108eaba0441fb45ec8e0073e945ae0ac1e138c933e4f2839816cd3198d7dd4d2</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786220171</t>
+          <t>1786225000</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1.900238</t>
+          <t>1.909308</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,12 +1083,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x0a5de930b5a6b8aca1699b666034af3891a3aa920021791d6d13e0297fb7903f</t>
+          <t>0x86f4b24298f4c19f9f856cb19af2a260f24dc2d391f252248469436057ea1d1a</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1098,12 +1098,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>49.99999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.6175</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Almirante Brown -1</t>
+          <t>Deportivo Moron -1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1123,27 +1123,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Deportivo Moron vs Acassuso</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Deportivo Moron</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Acassuso</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
+          <t>0xb61b063252c01d0525ae633a0276dc1830eabd418482fddec925fcbd602a2a75</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683452</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1168,17 +1168,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786218515</t>
+          <t>1786220171</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786298400</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>80.971644</t>
+          <t>1.900238</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,23 +1195,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x17d5a08f8fa305f31f27442393c64f497dd3893417da6e76c321c4c2a187320d</t>
+          <t>0x0a5de930b5a6b8aca1699b666034af3891a3aa920021791d6d13e0297fb7903f</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0x4a09916b1325Eed50eE8973B13742a205B0B7c7E</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>49.18897</t>
+          <t>49.99999</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4737</t>
+          <t>1.6175</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1219,7 +1223,11 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Almirante Brown -1</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -1272,7 +1280,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786218084</t>
+          <t>1786218515</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1282,7 +1290,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>103.82896</t>
+          <t>80.971644</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,28 +1307,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x56975f372357be259365cb7d2929c88d4fae157eea7a71d53d57cb234834f2ca</t>
+          <t>0x17d5a08f8fa305f31f27442393c64f497dd3893417da6e76c321c4c2a187320d</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>49.18897</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.4812</t>
+          <t>1.4737</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1331,27 +1339,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Club Atletico Mitre de Santiago del Estero vs Defensores de Belgrano Buenos Aires</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Club Atletico Mitre de Santiago del Estero</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Defensores de Belgrano Buenos Aires</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xa8ade64a3adb0ea38de67a61105ef31beb490d5a7287715b76ae124536d359cc</t>
+          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19683493</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1376,17 +1384,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786215674</t>
+          <t>1786218084</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2.077922</t>
+          <t>103.82896</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,7 +1411,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xff53df1f3446908699196d44fcdb8b39c1bd15c7ed519f0d730e55a51a6eb38f</t>
+          <t>0x56975f372357be259365cb7d2929c88d4fae157eea7a71d53d57cb234834f2ca</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1411,11 +1419,7 @@
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>1</t>
@@ -1423,19 +1427,15 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.3713</t>
+          <t>1.4812</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Almirante Brown</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -1443,27 +1443,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Club Atletico Mitre de Santiago del Estero vs Defensores de Belgrano Buenos Aires</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Club Atletico Mitre de Santiago del Estero</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Defensores de Belgrano Buenos Aires</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x63a8bf73c1084ef223fdd1096dccd16232e7a455fad77f7f0891be1588ebeb88</t>
+          <t>0xa8ade64a3adb0ea38de67a61105ef31beb490d5a7287715b76ae124536d359cc</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683493</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1488,17 +1488,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786215673</t>
+          <t>1786215674</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2.693603</t>
+          <t>2.077922</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1515,12 +1515,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x249d52552e7acb9f472d2a4c48ab754622ba572903281739a3e10b4d509dccb0</t>
+          <t>0xff53df1f3446908699196d44fcdb8b39c1bd15c7ed519f0d730e55a51a6eb38f</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1530,22 +1530,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.2288</t>
+          <t>1.3713</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Almirante Brown -1</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
+          <t>0x63a8bf73c1084ef223fdd1096dccd16232e7a455fad77f7f0891be1588ebeb88</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786214209</t>
+          <t>1786215673</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>6.295082</t>
+          <t>2.693603</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1627,12 +1627,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xf65c55196eeb0d21e7e3866ad26f8c3f2fee2aef273ddde5423e31fb40a51469</t>
+          <t>0x249d52552e7acb9f472d2a4c48ab754622ba572903281739a3e10b4d509dccb0</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1642,39 +1642,39 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>121.81</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.4363</t>
+          <t>1.2288</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Almirante Brown -1</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>Almirante Brown</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Almirante Brown</t>
-        </is>
-      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>Ciudad Bolivar</t>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x63a8bf73c1084ef223fdd1096dccd16232e7a455fad77f7f0891be1588ebeb88</t>
+          <t>0xa6a338c64f062bfd589e8d5d9cea45a27c9e64065f71f800e5966f81ce53c556</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786213844</t>
+          <t>1786214209</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>279.22063</t>
+          <t>6.295082</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1739,7 +1739,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x1bb20a2bf22e4fe06b44c06b9c2caa21f3f2a7c9d0cce1a2346f79e76022cd1f</t>
+          <t>0xf65c55196eeb0d21e7e3866ad26f8c3f2fee2aef273ddde5423e31fb40a51469</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>21.05</t>
+          <t>121.81</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Almirante Brown -0.5</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xfa00d2f0c7b5053ee336b303a0e7ad9cec0b8d539367773b7efee5c86cb2b59d</t>
+          <t>0x63a8bf73c1084ef223fdd1096dccd16232e7a455fad77f7f0891be1588ebeb88</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786213843</t>
+          <t>1786213844</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>48.252149</t>
+          <t>279.22063</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1851,7 +1851,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xc51052f8e449b4d56cc87b697bfc8eb0d3a88ae218dee1da3d725fa94163bc75</t>
+          <t>0x1bb20a2bf22e4fe06b44c06b9c2caa21f3f2a7c9d0cce1a2346f79e76022cd1f</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1859,28 +1859,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>77.29513</t>
+          <t>21.05</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2588</t>
+          <t>1.4363</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Almirante Brown -0.5</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>Almirante Brown vs Ciudad Bolivar</t>
@@ -1898,7 +1906,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xaa5316c6f6544d74142ad6db34a3745918f237ffb1a657e000693947e81b65d6</t>
+          <t>0xfa00d2f0c7b5053ee336b303a0e7ad9cec0b8d539367773b7efee5c86cb2b59d</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1928,7 +1936,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786212849</t>
+          <t>1786213843</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1938,7 +1946,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>298.72514</t>
+          <t>48.252149</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1955,7 +1963,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x0aeb4fe40f7d734cf244c144e6c064568b40b222193c9f93c641d1b31af3752e</t>
+          <t>0xc51052f8e449b4d56cc87b697bfc8eb0d3a88ae218dee1da3d725fa94163bc75</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1966,7 +1974,7 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>16.89162</t>
+          <t>77.29513</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2032,7 +2040,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786212805</t>
+          <t>1786212849</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2042,7 +2050,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>65.281623</t>
+          <t>298.72514</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2059,7 +2067,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x383b895a5fe529a887369a0f113c516fdc7f6125d54381acf9695997ef22d039</t>
+          <t>0x0aeb4fe40f7d734cf244c144e6c064568b40b222193c9f93c641d1b31af3752e</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2067,19 +2075,15 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>11.26905</t>
+          <t>16.89162</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.2588</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2087,26 +2091,22 @@
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>Almirante Brown</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Primera Nacional</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Almirante Brown</t>
-        </is>
-      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>Ciudad Bolivar</t>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786211779</t>
+          <t>1786212805</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>15.126242</t>
+          <t>65.281623</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2171,12 +2171,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xcfb6add6f8610a64ffc187beb9e16bf2bacb27b54a0f0aaefa6bfb437239b893</t>
+          <t>0x383b895a5fe529a887369a0f113c516fdc7f6125d54381acf9695997ef22d039</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>24.89998</t>
+          <t>11.26905</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786211777</t>
+          <t>1786211779</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>33.422792</t>
+          <t>15.126242</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2283,12 +2283,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xd41652604437a4e92e0d78b653d4d49d8dedd2e153d1340dad89b9b93e182a48</t>
+          <t>0xcfb6add6f8610a64ffc187beb9e16bf2bacb27b54a0f0aaefa6bfb437239b893</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2298,22 +2298,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>24.89998</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4163</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Primera Nacional</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Atl. Rafaela</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2323,27 +2323,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Atl. Rafaela vs Chacarita Juniors</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Atl. Rafaela</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Chacarita Juniors</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xe738e9ba05492fab73eaaf6da211b84caadc72b08b26f1cd30fa8737e283bb44</t>
+          <t>0xaa5316c6f6544d74142ad6db34a3745918f237ffb1a657e000693947e81b65d6</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19683450</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2368,17 +2368,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786211028</t>
+          <t>1786211777</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786215600</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2.402402</t>
+          <t>33.422792</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2395,31 +2395,39 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x562fd7c6419c807ed04d3cacac95f861805f96704bd535e265399fb9d2c2b609</t>
+          <t>0xd41652604437a4e92e0d78b653d4d49d8dedd2e153d1340dad89b9b93e182a48</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.32</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.405</t>
+          <t>1.4163</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Atl. Rafaela</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2427,27 +2435,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
+          <t>Atl. Rafaela vs Chacarita Juniors</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros</t>
+          <t>Atl. Rafaela</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Chacarita Juniors</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
+          <t>0xe738e9ba05492fab73eaaf6da211b84caadc72b08b26f1cd30fa8737e283bb44</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19683453</t>
+          <t>L19683450</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2472,17 +2480,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786210845</t>
+          <t>1786211028</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786215600</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.135802</t>
+          <t>2.402402</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2499,39 +2507,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x0bb7a6822220bf40d7b279f99a54f46025f393ba95bb38b6d6dc98192886b3ed</t>
+          <t>0x562fd7c6419c807ed04d3cacac95f861805f96704bd535e265399fb9d2c2b609</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.99999</t>
+          <t>5.32</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.5513</t>
+          <t>1.405</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Agropecuario</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2539,27 +2539,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Agropecuario vs Atletico Guemes</t>
+          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Agropecuario</t>
+          <t>Estudiantes de Caseros</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Atletico Guemes</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xae66c7fab3c9c76fbc29d9e9778ef4845d8a6b8d092cff34320f100020113c49</t>
+          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19683451</t>
+          <t>L19683453</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786205982</t>
+          <t>1786210845</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1.814041</t>
+          <t>13.135802</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2611,7 +2611,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xe17b2546f4b90c8647ba975c279e39dec1fda5a003adfb8a2b39bb12a3519b10</t>
+          <t>0x0bb7a6822220bf40d7b279f99a54f46025f393ba95bb38b6d6dc98192886b3ed</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2626,12 +2626,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.99999</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.3613</t>
+          <t>1.5513</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2641,7 +2641,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Agropecuario</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2651,27 +2651,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Agropecuario vs Atletico Guemes</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Agropecuario</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Atletico Guemes</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xd5906ce08d61f7c5ee45fcebd2c8baeed5558387398ea332817a4b632f439b6d</t>
+          <t>0xae66c7fab3c9c76fbc29d9e9778ef4845d8a6b8d092cff34320f100020113c49</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683451</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786205963</t>
+          <t>1786205982</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2.768166</t>
+          <t>1.814041</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2723,7 +2723,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xcfe218822e89cbef5841f3045f551cc65acf353d8e240f943e2b61c54ea79a68</t>
+          <t>0xe17b2546f4b90c8647ba975c279e39dec1fda5a003adfb8a2b39bb12a3519b10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.3337</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2763,27 +2763,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xf238b96ec9e2421db79973de945f1fc0c3f8bb99c31cda32d011ebaabfd2db86</t>
+          <t>0xd5906ce08d61f7c5ee45fcebd2c8baeed5558387398ea332817a4b632f439b6d</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19683453</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786205938</t>
+          <t>1786205963</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2.996255</t>
+          <t>2.768166</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2835,31 +2835,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x1b9fcb29010a212f74af57040114154e78748f06a4d826be4397ddadb45ac31b</t>
+          <t>0xcfe218822e89cbef5841f3045f551cc65acf353d8e240f943e2b61c54ea79a68</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
+          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>21.69</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.3337</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -2867,27 +2875,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Estudiantes de Caseros</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
+          <t>0xf238b96ec9e2421db79973de945f1fc0c3f8bb99c31cda32d011ebaabfd2db86</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683453</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2912,7 +2920,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786190525</t>
+          <t>1786205938</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2922,7 +2930,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>48.066482</t>
+          <t>2.996255</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2939,23 +2947,23 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x3177792dd6a7185e37ae06612104cf5a35d137d7f535a889a83a7e9b7c174506</t>
+          <t>0x1b9fcb29010a212f74af57040114154e78748f06a4d826be4397ddadb45ac31b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>18.35495</t>
+          <t>21.69</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.4963</t>
+          <t>1.4512</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3016,7 +3024,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786190491</t>
+          <t>1786190525</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3026,7 +3034,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>36.987305</t>
+          <t>48.066482</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3043,7 +3051,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x54ed4ee2a6ebdab49498137f1accea542ead806f21430a0a771cc4872a044e43</t>
+          <t>0x3177792dd6a7185e37ae06612104cf5a35d137d7f535a889a83a7e9b7c174506</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3051,19 +3059,15 @@
           <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>20.10741</t>
+          <t>18.35495</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.4963</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3071,11 +3075,7 @@
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786190485</t>
+          <t>1786190491</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>36.979145</t>
+          <t>36.987305</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3155,23 +3155,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x544fe5c906328d009917b591611ff3438cef85f8b42d9f67732cbbd5eabbb8dd</t>
+          <t>0x54ed4ee2a6ebdab49498137f1accea542ead806f21430a0a771cc4872a044e43</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>21.69</t>
+          <t>20.10741</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3179,7 +3183,11 @@
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
@@ -3242,7 +3250,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>48.066482</t>
+          <t>36.979145</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3259,7 +3267,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xb2f3ea804e1760a01d3a93678f0e2119f1ea2a9db0dc4711a06cc7bcba42b0c2</t>
+          <t>0x544fe5c906328d009917b591611ff3438cef85f8b42d9f67732cbbd5eabbb8dd</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3270,12 +3278,12 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>17.47</t>
+          <t>21.69</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.405</t>
+          <t>1.4512</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3291,27 +3299,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Estudiantes de Caseros</t>
+          <t>Almirante Brown</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Ciudad Bolivar</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
+          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19683453</t>
+          <t>L19683447</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3336,7 +3344,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786190461</t>
+          <t>1786190485</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3346,7 +3354,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>43.135802</t>
+          <t>48.066482</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3363,7 +3371,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xa7eafbb77d425fc2347b4ee3e4f4e1b85f6d0f81420605db76ebfeeaa793a428</t>
+          <t>0xb2f3ea804e1760a01d3a93678f0e2119f1ea2a9db0dc4711a06cc7bcba42b0c2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3374,12 +3382,12 @@
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>21.69</t>
+          <t>17.47</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.405</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3395,27 +3403,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Almirante Brown vs Ciudad Bolivar</t>
+          <t>Estudiantes de Caseros vs Deportivo Madryn</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Almirante Brown</t>
+          <t>Estudiantes de Caseros</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Ciudad Bolivar</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
+          <t>0xd61509e26f8645bb9780672f942c72c4b7dab577c2a01f04e1e09bce9b828765</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19683447</t>
+          <t>L19683453</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3440,7 +3448,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786190458</t>
+          <t>1786190461</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3450,7 +3458,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>48.066482</t>
+          <t>43.135802</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3467,110 +3475,214 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>0xa7eafbb77d425fc2347b4ee3e4f4e1b85f6d0f81420605db76ebfeeaa793a428</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>21.69</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Primera Nacional</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Almirante Brown vs Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Almirante Brown</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Ciudad Bolivar</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0xbbcaa253cd967fbf933ff0d87a6f9744cafec0ed59dad5f1f76332aab01a3fa5</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>L19683447</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1786190458</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>48.066482</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>0x5c5b512ea725fac30531bf5fe91f34f3ccc0eeff23890c18f25c3f329007c589</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>1.3638</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>Primera Nacional</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>Almirante Brown vs Ciudad Bolivar</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>Almirante Brown</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>Ciudad Bolivar</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>0xd5906ce08d61f7c5ee45fcebd2c8baeed5558387398ea332817a4b632f439b6d</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>L19683447</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
         <is>
           <t>1786125660</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="S30" t="inlineStr">
         <is>
           <t>1786212000</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr">
+      <c r="T30" t="inlineStr">
         <is>
           <t>2.749141</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="U30" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr">
+      <c r="V30" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>